<commit_message>
Did some more work
</commit_message>
<xml_diff>
--- a/BoM.xlsx
+++ b/BoM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/matthew_mcinnes_swaney_npl_co_uk/Documents/Documents/J/SLSS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{93ED6D48-6C45-4EA7-9344-3347BCEAFEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D28EED71-38E4-400B-8EB5-F8F4B3C30805}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{93ED6D48-6C45-4EA7-9344-3347BCEAFEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB4D96D2-0EA5-4A0A-BC55-D2146005661E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -129,6 +129,15 @@
   </si>
   <si>
     <t>https://uk.rs-online.com/web/p/potentiometers/8427002?gb=s</t>
+  </si>
+  <si>
+    <t>SFH3501-16L | SPREADFAST Heatsink, Universal Square Alu, 35 x 35 x 16mm | RS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heatsink </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peltier </t>
   </si>
 </sst>
 </file>
@@ -703,7 +712,23 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="2:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" display="https://cpc.farnell.com/mean-well/rs-25-5/psu-enclosed-5v-25w/dp/PW01558?st=5v%205a%20power%20supplies" xr:uid="{2C210EEA-7D0A-48FE-8CEC-1DC95A3D182C}"/>
@@ -716,6 +741,7 @@
     <hyperlink ref="G7" r:id="rId8" xr:uid="{FDE6AEF3-69D3-416F-A56A-1007D8E1F2EA}"/>
     <hyperlink ref="H7" r:id="rId9" xr:uid="{33A00EBA-6D17-45EC-B033-B94BB4B69474}"/>
     <hyperlink ref="F11" r:id="rId10" xr:uid="{1717598A-4686-441A-9EF8-DAB2430DA4C2}"/>
+    <hyperlink ref="F12" r:id="rId11" display="https://uk.rs-online.com/web/p/heatsinks/1846721?searchId=099ba976-54d0-4342-b192-1b402f10c554" xr:uid="{99CAD027-3F84-411B-979C-FA6BFBFA6BC4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>